<commit_message>
Fix import excel role sarpras
</commit_message>
<xml_diff>
--- a/public/template-buku-alat.xlsx
+++ b/public/template-buku-alat.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24701"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25427"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\diakademik\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{827BE3DE-21BF-4BE6-B007-FF27138D5798}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{540226E1-E63C-4131-A828-5272C18A0A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{11918E53-3184-4236-A3F0-F69A85483F71}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Jenis Buku Atau Alat</t>
   </si>
@@ -68,6 +68,15 @@
   </si>
   <si>
     <t>Kondisi Rusak</t>
+  </si>
+  <si>
+    <t>Tingkat Pendidikan</t>
+  </si>
+  <si>
+    <t>Mata Pelajaran</t>
+  </si>
+  <si>
+    <t>Tata Boga</t>
   </si>
 </sst>
 </file>
@@ -427,20 +436,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DE9CB0C-BCF5-43F1-AE75-0C0F9D924117}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="17.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="18.6328125" customWidth="1"/>
+    <col min="5" max="5" width="17.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -448,47 +458,59 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>10</v>
       </c>
       <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="2">
+      <c r="F2" s="2">
         <v>43831</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>10</v>
       </c>
-      <c r="F2">
+      <c r="H2">
         <v>9</v>
       </c>
-      <c r="G2">
+      <c r="I2">
         <v>1</v>
       </c>
-      <c r="H2" t="s">
+      <c r="J2" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>